<commit_message>
subir fase 5, errores en documentos, crear pruebas, agregar profesor
</commit_message>
<xml_diff>
--- a/public/docs/fase1/product_backlog_ajuptel.xlsx
+++ b/public/docs/fase1/product_backlog_ajuptel.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="BACKLOG" sheetId="1" state="visible" r:id="rId3"/>
@@ -2453,7 +2453,7 @@
     <t xml:space="preserve">Actividades/Historias</t>
   </si>
   <si>
-    <t xml:space="preserve">No se estiman puntos de historias</t>
+    <t xml:space="preserve">Observaciones</t>
   </si>
   <si>
     <t xml:space="preserve">Fase de Preparación Técnica </t>
@@ -2909,7 +2909,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="@"/>
   </numFmts>
-  <fonts count="17">
+  <fonts count="16">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2996,12 +2996,6 @@
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
@@ -3174,7 +3168,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="56">
+  <cellXfs count="55">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -3263,10 +3257,6 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="5" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -3299,11 +3289,11 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3327,7 +3317,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3387,7 +3377,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3619,9 +3609,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
-      <xdr:colOff>1425600</xdr:colOff>
+      <xdr:colOff>1425240</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>857880</xdr:rowOff>
+      <xdr:rowOff>857520</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -3636,7 +3626,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="10617120" cy="857880"/>
+          <a:ext cx="10616760" cy="857520"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3663,9 +3653,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>2520000</xdr:colOff>
+      <xdr:colOff>2519640</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>768240</xdr:rowOff>
+      <xdr:rowOff>767880</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -3680,7 +3670,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="26640" y="195480"/>
-          <a:ext cx="7426080" cy="572760"/>
+          <a:ext cx="7425720" cy="572400"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3707,9 +3697,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>1042920</xdr:colOff>
+      <xdr:colOff>1042560</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>654480</xdr:rowOff>
+      <xdr:rowOff>654120</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -3724,7 +3714,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="95400"/>
-          <a:ext cx="6611400" cy="559080"/>
+          <a:ext cx="6611040" cy="558720"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -4236,7 +4226,7 @@
       <c r="M19" s="21" t="n">
         <v>1</v>
       </c>
-      <c r="N19" s="22" t="s">
+      <c r="N19" s="21" t="s">
         <v>45</v>
       </c>
       <c r="O19" s="21"/>
@@ -4311,7 +4301,7 @@
       <c r="M22" s="21" t="n">
         <v>1</v>
       </c>
-      <c r="N22" s="22" t="s">
+      <c r="N22" s="21" t="s">
         <v>45</v>
       </c>
       <c r="O22" s="21"/>
@@ -4356,7 +4346,7 @@
       <c r="O24" s="21"/>
     </row>
     <row r="25" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="23" t="s">
+      <c r="A25" s="22" t="s">
         <v>62</v>
       </c>
       <c r="B25" s="17" t="s">
@@ -4395,13 +4385,13 @@
       <c r="M25" s="21" t="n">
         <v>2</v>
       </c>
-      <c r="N25" s="22" t="s">
+      <c r="N25" s="21" t="s">
         <v>45</v>
       </c>
       <c r="O25" s="21"/>
     </row>
     <row r="26" customFormat="false" ht="94.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="23"/>
+      <c r="A26" s="22"/>
       <c r="B26" s="17"/>
       <c r="C26" s="17"/>
       <c r="D26" s="19"/>
@@ -4420,7 +4410,7 @@
       <c r="O26" s="21"/>
     </row>
     <row r="27" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="23"/>
+      <c r="A27" s="22"/>
       <c r="B27" s="17"/>
       <c r="C27" s="17"/>
       <c r="D27" s="19"/>
@@ -4439,7 +4429,7 @@
       <c r="O27" s="21"/>
     </row>
     <row r="28" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="23"/>
+      <c r="A28" s="22"/>
       <c r="B28" s="17"/>
       <c r="C28" s="17"/>
       <c r="D28" s="19"/>
@@ -4458,7 +4448,7 @@
       <c r="O28" s="21"/>
     </row>
     <row r="29" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="23"/>
+      <c r="A29" s="22"/>
       <c r="B29" s="17"/>
       <c r="C29" s="17"/>
       <c r="D29" s="19"/>
@@ -4477,7 +4467,7 @@
       <c r="O29" s="21"/>
     </row>
     <row r="30" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="23"/>
+      <c r="A30" s="22"/>
       <c r="B30" s="17"/>
       <c r="C30" s="17"/>
       <c r="D30" s="19"/>
@@ -4514,7 +4504,7 @@
       <c r="O30" s="21"/>
     </row>
     <row r="31" customFormat="false" ht="50.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="23"/>
+      <c r="A31" s="22"/>
       <c r="B31" s="17"/>
       <c r="C31" s="17"/>
       <c r="D31" s="19"/>
@@ -4533,7 +4523,7 @@
       <c r="O31" s="21"/>
     </row>
     <row r="32" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="23"/>
+      <c r="A32" s="22"/>
       <c r="B32" s="17"/>
       <c r="C32" s="17"/>
       <c r="D32" s="19"/>
@@ -4541,7 +4531,7 @@
       <c r="F32" s="19"/>
       <c r="G32" s="19"/>
       <c r="H32" s="19"/>
-      <c r="I32" s="24" t="s">
+      <c r="I32" s="23" t="s">
         <v>80</v>
       </c>
       <c r="J32" s="21"/>
@@ -4552,7 +4542,7 @@
       <c r="O32" s="21"/>
     </row>
     <row r="33" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="23"/>
+      <c r="A33" s="22"/>
       <c r="B33" s="17"/>
       <c r="C33" s="17"/>
       <c r="D33" s="19"/>
@@ -4583,13 +4573,13 @@
       <c r="M33" s="21" t="n">
         <v>2</v>
       </c>
-      <c r="N33" s="22" t="s">
+      <c r="N33" s="21" t="s">
         <v>45</v>
       </c>
       <c r="O33" s="21"/>
     </row>
     <row r="34" customFormat="false" ht="49.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="23"/>
+      <c r="A34" s="22"/>
       <c r="B34" s="17"/>
       <c r="C34" s="17"/>
       <c r="D34" s="19"/>
@@ -4597,7 +4587,7 @@
       <c r="F34" s="19"/>
       <c r="G34" s="19"/>
       <c r="H34" s="19"/>
-      <c r="I34" s="24" t="s">
+      <c r="I34" s="23" t="s">
         <v>85</v>
       </c>
       <c r="J34" s="21"/>
@@ -4608,7 +4598,7 @@
       <c r="O34" s="21"/>
     </row>
     <row r="35" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="23"/>
+      <c r="A35" s="22"/>
       <c r="B35" s="17"/>
       <c r="C35" s="17"/>
       <c r="D35" s="19"/>
@@ -4616,7 +4606,7 @@
       <c r="F35" s="19"/>
       <c r="G35" s="19"/>
       <c r="H35" s="19"/>
-      <c r="I35" s="24" t="s">
+      <c r="I35" s="23" t="s">
         <v>86</v>
       </c>
       <c r="J35" s="21"/>
@@ -4627,7 +4617,7 @@
       <c r="O35" s="21"/>
     </row>
     <row r="36" customFormat="false" ht="49.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="23"/>
+      <c r="A36" s="22"/>
       <c r="B36" s="17"/>
       <c r="C36" s="17"/>
       <c r="D36" s="19"/>
@@ -4643,7 +4633,7 @@
       <c r="H36" s="19" t="s">
         <v>90</v>
       </c>
-      <c r="I36" s="24" t="s">
+      <c r="I36" s="23" t="s">
         <v>91</v>
       </c>
       <c r="J36" s="21" t="s">
@@ -4658,13 +4648,13 @@
       <c r="M36" s="21" t="n">
         <v>2</v>
       </c>
-      <c r="N36" s="22" t="s">
+      <c r="N36" s="21" t="s">
         <v>45</v>
       </c>
       <c r="O36" s="21"/>
     </row>
     <row r="37" customFormat="false" ht="77.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="23"/>
+      <c r="A37" s="22"/>
       <c r="B37" s="17"/>
       <c r="C37" s="17"/>
       <c r="D37" s="19"/>
@@ -4672,7 +4662,7 @@
       <c r="F37" s="19"/>
       <c r="G37" s="19"/>
       <c r="H37" s="19"/>
-      <c r="I37" s="24" t="s">
+      <c r="I37" s="23" t="s">
         <v>92</v>
       </c>
       <c r="J37" s="21"/>
@@ -4683,7 +4673,7 @@
       <c r="O37" s="21"/>
     </row>
     <row r="38" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="23"/>
+      <c r="A38" s="22"/>
       <c r="B38" s="17"/>
       <c r="C38" s="17"/>
       <c r="D38" s="19"/>
@@ -4691,7 +4681,7 @@
       <c r="F38" s="19"/>
       <c r="G38" s="19"/>
       <c r="H38" s="19"/>
-      <c r="I38" s="24" t="s">
+      <c r="I38" s="23" t="s">
         <v>93</v>
       </c>
       <c r="J38" s="21"/>
@@ -4702,7 +4692,7 @@
       <c r="O38" s="21"/>
     </row>
     <row r="39" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="25" t="s">
+      <c r="A39" s="24" t="s">
         <v>94</v>
       </c>
       <c r="B39" s="19" t="s">
@@ -4741,13 +4731,13 @@
       <c r="M39" s="21" t="n">
         <v>3</v>
       </c>
-      <c r="N39" s="22" t="s">
+      <c r="N39" s="21" t="s">
         <v>45</v>
       </c>
       <c r="O39" s="21"/>
     </row>
     <row r="40" customFormat="false" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="25"/>
+      <c r="A40" s="24"/>
       <c r="B40" s="19"/>
       <c r="C40" s="19"/>
       <c r="D40" s="19"/>
@@ -4755,7 +4745,7 @@
       <c r="F40" s="19"/>
       <c r="G40" s="19"/>
       <c r="H40" s="19"/>
-      <c r="I40" s="24" t="s">
+      <c r="I40" s="23" t="s">
         <v>102</v>
       </c>
       <c r="J40" s="21"/>
@@ -4766,7 +4756,7 @@
       <c r="O40" s="21"/>
     </row>
     <row r="41" customFormat="false" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="25"/>
+      <c r="A41" s="24"/>
       <c r="B41" s="19"/>
       <c r="C41" s="19"/>
       <c r="D41" s="19"/>
@@ -4774,7 +4764,7 @@
       <c r="F41" s="19"/>
       <c r="G41" s="19"/>
       <c r="H41" s="19"/>
-      <c r="I41" s="24" t="s">
+      <c r="I41" s="23" t="s">
         <v>103</v>
       </c>
       <c r="J41" s="21"/>
@@ -4785,7 +4775,7 @@
       <c r="O41" s="21"/>
     </row>
     <row r="42" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="25"/>
+      <c r="A42" s="24"/>
       <c r="B42" s="19"/>
       <c r="C42" s="19"/>
       <c r="D42" s="19"/>
@@ -4816,13 +4806,13 @@
       <c r="M42" s="21" t="n">
         <v>3</v>
       </c>
-      <c r="N42" s="22" t="s">
+      <c r="N42" s="21" t="s">
         <v>45</v>
       </c>
       <c r="O42" s="21"/>
     </row>
     <row r="43" customFormat="false" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="25"/>
+      <c r="A43" s="24"/>
       <c r="B43" s="19"/>
       <c r="C43" s="19"/>
       <c r="D43" s="19"/>
@@ -4830,7 +4820,7 @@
       <c r="F43" s="19"/>
       <c r="G43" s="19"/>
       <c r="H43" s="19"/>
-      <c r="I43" s="24" t="s">
+      <c r="I43" s="23" t="s">
         <v>108</v>
       </c>
       <c r="J43" s="21"/>
@@ -4841,7 +4831,7 @@
       <c r="O43" s="21"/>
     </row>
     <row r="44" customFormat="false" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="25"/>
+      <c r="A44" s="24"/>
       <c r="B44" s="19"/>
       <c r="C44" s="19"/>
       <c r="D44" s="19"/>
@@ -4849,7 +4839,7 @@
       <c r="F44" s="19"/>
       <c r="G44" s="19"/>
       <c r="H44" s="19"/>
-      <c r="I44" s="24" t="s">
+      <c r="I44" s="23" t="s">
         <v>109</v>
       </c>
       <c r="J44" s="21"/>
@@ -4860,7 +4850,7 @@
       <c r="O44" s="21"/>
     </row>
     <row r="45" customFormat="false" ht="39.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A45" s="25"/>
+      <c r="A45" s="24"/>
       <c r="B45" s="19"/>
       <c r="C45" s="19"/>
       <c r="D45" s="19"/>
@@ -4891,13 +4881,13 @@
       <c r="M45" s="21" t="n">
         <v>3</v>
       </c>
-      <c r="N45" s="22" t="s">
+      <c r="N45" s="21" t="s">
         <v>45</v>
       </c>
       <c r="O45" s="21"/>
     </row>
     <row r="46" customFormat="false" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="25"/>
+      <c r="A46" s="24"/>
       <c r="B46" s="19"/>
       <c r="C46" s="19"/>
       <c r="D46" s="19"/>
@@ -4916,7 +4906,7 @@
       <c r="O46" s="21"/>
     </row>
     <row r="47" customFormat="false" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="25"/>
+      <c r="A47" s="24"/>
       <c r="B47" s="19"/>
       <c r="C47" s="19"/>
       <c r="D47" s="19"/>
@@ -4935,7 +4925,7 @@
       <c r="O47" s="21"/>
     </row>
     <row r="48" customFormat="false" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="25"/>
+      <c r="A48" s="24"/>
       <c r="B48" s="19"/>
       <c r="C48" s="19"/>
       <c r="D48" s="19"/>
@@ -4954,7 +4944,7 @@
       <c r="O48" s="21"/>
     </row>
     <row r="49" customFormat="false" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="25"/>
+      <c r="A49" s="24"/>
       <c r="B49" s="19"/>
       <c r="C49" s="19"/>
       <c r="D49" s="19"/>
@@ -4973,7 +4963,7 @@
       <c r="O49" s="21"/>
     </row>
     <row r="50" customFormat="false" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="25"/>
+      <c r="A50" s="24"/>
       <c r="B50" s="19"/>
       <c r="C50" s="19"/>
       <c r="D50" s="19"/>
@@ -4992,7 +4982,7 @@
       <c r="O50" s="21"/>
     </row>
     <row r="51" customFormat="false" ht="39.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A51" s="25"/>
+      <c r="A51" s="24"/>
       <c r="B51" s="19"/>
       <c r="C51" s="19"/>
       <c r="D51" s="19"/>
@@ -5008,7 +4998,7 @@
       <c r="H51" s="19" t="s">
         <v>122</v>
       </c>
-      <c r="I51" s="24" t="s">
+      <c r="I51" s="23" t="s">
         <v>123</v>
       </c>
       <c r="J51" s="21" t="s">
@@ -5023,13 +5013,13 @@
       <c r="M51" s="21" t="n">
         <v>3</v>
       </c>
-      <c r="N51" s="22" t="s">
+      <c r="N51" s="21" t="s">
         <v>45</v>
       </c>
       <c r="O51" s="21"/>
     </row>
     <row r="52" customFormat="false" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="25"/>
+      <c r="A52" s="24"/>
       <c r="B52" s="19"/>
       <c r="C52" s="19"/>
       <c r="D52" s="19"/>
@@ -5037,7 +5027,7 @@
       <c r="F52" s="19"/>
       <c r="G52" s="19"/>
       <c r="H52" s="19"/>
-      <c r="I52" s="24" t="s">
+      <c r="I52" s="23" t="s">
         <v>125</v>
       </c>
       <c r="J52" s="21"/>
@@ -5048,7 +5038,7 @@
       <c r="O52" s="21"/>
     </row>
     <row r="53" customFormat="false" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="25"/>
+      <c r="A53" s="24"/>
       <c r="B53" s="19"/>
       <c r="C53" s="19"/>
       <c r="D53" s="19"/>
@@ -5056,7 +5046,7 @@
       <c r="F53" s="19"/>
       <c r="G53" s="19"/>
       <c r="H53" s="19"/>
-      <c r="I53" s="24" t="s">
+      <c r="I53" s="23" t="s">
         <v>126</v>
       </c>
       <c r="J53" s="21"/>
@@ -5067,7 +5057,7 @@
       <c r="O53" s="21"/>
     </row>
     <row r="54" customFormat="false" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="25"/>
+      <c r="A54" s="24"/>
       <c r="B54" s="19"/>
       <c r="C54" s="19"/>
       <c r="D54" s="19"/>
@@ -5075,7 +5065,7 @@
       <c r="F54" s="19"/>
       <c r="G54" s="19"/>
       <c r="H54" s="19"/>
-      <c r="I54" s="24" t="s">
+      <c r="I54" s="23" t="s">
         <v>127</v>
       </c>
       <c r="J54" s="21"/>
@@ -5086,7 +5076,7 @@
       <c r="O54" s="21"/>
     </row>
     <row r="55" customFormat="false" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="25"/>
+      <c r="A55" s="24"/>
       <c r="B55" s="19"/>
       <c r="C55" s="19"/>
       <c r="D55" s="19"/>
@@ -5094,7 +5084,7 @@
       <c r="F55" s="19"/>
       <c r="G55" s="19"/>
       <c r="H55" s="19"/>
-      <c r="I55" s="24" t="s">
+      <c r="I55" s="23" t="s">
         <v>128</v>
       </c>
       <c r="J55" s="21"/>
@@ -5105,7 +5095,7 @@
       <c r="O55" s="21"/>
     </row>
     <row r="56" customFormat="false" ht="39.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A56" s="26" t="s">
+      <c r="A56" s="25" t="s">
         <v>129</v>
       </c>
       <c r="B56" s="19" t="s">
@@ -5144,13 +5134,13 @@
       <c r="M56" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="N56" s="22" t="s">
+      <c r="N56" s="21" t="s">
         <v>45</v>
       </c>
       <c r="O56" s="21"/>
     </row>
     <row r="57" customFormat="false" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="26"/>
+      <c r="A57" s="25"/>
       <c r="B57" s="19"/>
       <c r="C57" s="19"/>
       <c r="D57" s="19"/>
@@ -5158,7 +5148,7 @@
       <c r="F57" s="19"/>
       <c r="G57" s="19"/>
       <c r="H57" s="19"/>
-      <c r="I57" s="24" t="s">
+      <c r="I57" s="23" t="s">
         <v>138</v>
       </c>
       <c r="J57" s="21"/>
@@ -5169,7 +5159,7 @@
       <c r="O57" s="21"/>
     </row>
     <row r="58" customFormat="false" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="26"/>
+      <c r="A58" s="25"/>
       <c r="B58" s="19"/>
       <c r="C58" s="19"/>
       <c r="D58" s="19"/>
@@ -5177,7 +5167,7 @@
       <c r="F58" s="19"/>
       <c r="G58" s="19"/>
       <c r="H58" s="19"/>
-      <c r="I58" s="24" t="s">
+      <c r="I58" s="23" t="s">
         <v>139</v>
       </c>
       <c r="J58" s="21"/>
@@ -5188,7 +5178,7 @@
       <c r="O58" s="21"/>
     </row>
     <row r="59" customFormat="false" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="26"/>
+      <c r="A59" s="25"/>
       <c r="B59" s="19"/>
       <c r="C59" s="19"/>
       <c r="D59" s="19"/>
@@ -5196,7 +5186,7 @@
       <c r="F59" s="19"/>
       <c r="G59" s="19"/>
       <c r="H59" s="19"/>
-      <c r="I59" s="24" t="s">
+      <c r="I59" s="23" t="s">
         <v>140</v>
       </c>
       <c r="J59" s="21"/>
@@ -5207,7 +5197,7 @@
       <c r="O59" s="21"/>
     </row>
     <row r="60" customFormat="false" ht="39.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A60" s="26"/>
+      <c r="A60" s="25"/>
       <c r="B60" s="19"/>
       <c r="C60" s="19"/>
       <c r="D60" s="19"/>
@@ -5238,13 +5228,13 @@
       <c r="M60" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="N60" s="22" t="s">
+      <c r="N60" s="21" t="s">
         <v>45</v>
       </c>
       <c r="O60" s="21"/>
     </row>
     <row r="61" customFormat="false" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="26"/>
+      <c r="A61" s="25"/>
       <c r="B61" s="19"/>
       <c r="C61" s="19"/>
       <c r="D61" s="19"/>
@@ -5252,7 +5242,7 @@
       <c r="F61" s="19"/>
       <c r="G61" s="19"/>
       <c r="H61" s="19"/>
-      <c r="I61" s="24" t="s">
+      <c r="I61" s="23" t="s">
         <v>147</v>
       </c>
       <c r="J61" s="21"/>
@@ -5263,7 +5253,7 @@
       <c r="O61" s="21"/>
     </row>
     <row r="62" customFormat="false" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="26"/>
+      <c r="A62" s="25"/>
       <c r="B62" s="19"/>
       <c r="C62" s="19"/>
       <c r="D62" s="19"/>
@@ -5271,7 +5261,7 @@
       <c r="F62" s="19"/>
       <c r="G62" s="19"/>
       <c r="H62" s="19"/>
-      <c r="I62" s="24" t="s">
+      <c r="I62" s="23" t="s">
         <v>148</v>
       </c>
       <c r="J62" s="21"/>
@@ -5282,7 +5272,7 @@
       <c r="O62" s="21"/>
     </row>
     <row r="63" customFormat="false" ht="39.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A63" s="27" t="s">
+      <c r="A63" s="26" t="s">
         <v>149</v>
       </c>
       <c r="B63" s="19" t="s">
@@ -5321,13 +5311,13 @@
       <c r="M63" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="N63" s="22" t="s">
+      <c r="N63" s="21" t="s">
         <v>45</v>
       </c>
       <c r="O63" s="21"/>
     </row>
     <row r="64" customFormat="false" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A64" s="27"/>
+      <c r="A64" s="26"/>
       <c r="B64" s="19"/>
       <c r="C64" s="19"/>
       <c r="D64" s="19"/>
@@ -5335,7 +5325,7 @@
       <c r="F64" s="19"/>
       <c r="G64" s="19"/>
       <c r="H64" s="19"/>
-      <c r="I64" s="24" t="s">
+      <c r="I64" s="23" t="s">
         <v>159</v>
       </c>
       <c r="J64" s="21"/>
@@ -5346,7 +5336,7 @@
       <c r="O64" s="21"/>
     </row>
     <row r="65" customFormat="false" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="27"/>
+      <c r="A65" s="26"/>
       <c r="B65" s="19"/>
       <c r="C65" s="19"/>
       <c r="D65" s="19"/>
@@ -5354,7 +5344,7 @@
       <c r="F65" s="19"/>
       <c r="G65" s="19"/>
       <c r="H65" s="19"/>
-      <c r="I65" s="24" t="s">
+      <c r="I65" s="23" t="s">
         <v>160</v>
       </c>
       <c r="J65" s="21"/>
@@ -5365,7 +5355,7 @@
       <c r="O65" s="21"/>
     </row>
     <row r="66" customFormat="false" ht="39.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A66" s="27"/>
+      <c r="A66" s="26"/>
       <c r="B66" s="19"/>
       <c r="C66" s="19"/>
       <c r="D66" s="19"/>
@@ -5396,13 +5386,13 @@
       <c r="M66" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="N66" s="22" t="s">
+      <c r="N66" s="21" t="s">
         <v>45</v>
       </c>
       <c r="O66" s="21"/>
     </row>
     <row r="67" customFormat="false" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="27"/>
+      <c r="A67" s="26"/>
       <c r="B67" s="19"/>
       <c r="C67" s="19"/>
       <c r="D67" s="19"/>
@@ -5410,7 +5400,7 @@
       <c r="F67" s="19"/>
       <c r="G67" s="19"/>
       <c r="H67" s="19"/>
-      <c r="I67" s="24" t="s">
+      <c r="I67" s="23" t="s">
         <v>165</v>
       </c>
       <c r="J67" s="21"/>
@@ -5421,7 +5411,7 @@
       <c r="O67" s="21"/>
     </row>
     <row r="68" customFormat="false" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A68" s="27"/>
+      <c r="A68" s="26"/>
       <c r="B68" s="19"/>
       <c r="C68" s="19"/>
       <c r="D68" s="19"/>
@@ -5429,7 +5419,7 @@
       <c r="F68" s="19"/>
       <c r="G68" s="19"/>
       <c r="H68" s="19"/>
-      <c r="I68" s="24" t="s">
+      <c r="I68" s="23" t="s">
         <v>166</v>
       </c>
       <c r="J68" s="21"/>
@@ -5440,7 +5430,7 @@
       <c r="O68" s="21"/>
     </row>
     <row r="69" customFormat="false" ht="39.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A69" s="28" t="s">
+      <c r="A69" s="27" t="s">
         <v>167</v>
       </c>
       <c r="B69" s="19" t="s">
@@ -5479,13 +5469,13 @@
       <c r="M69" s="21" t="n">
         <v>5</v>
       </c>
-      <c r="N69" s="22" t="s">
+      <c r="N69" s="21" t="s">
         <v>45</v>
       </c>
       <c r="O69" s="21"/>
     </row>
     <row r="70" customFormat="false" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A70" s="28"/>
+      <c r="A70" s="27"/>
       <c r="B70" s="19"/>
       <c r="C70" s="19"/>
       <c r="D70" s="19"/>
@@ -5504,7 +5494,7 @@
       <c r="O70" s="21"/>
     </row>
     <row r="71" customFormat="false" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A71" s="28"/>
+      <c r="A71" s="27"/>
       <c r="B71" s="19"/>
       <c r="C71" s="19"/>
       <c r="D71" s="19"/>
@@ -5523,7 +5513,7 @@
       <c r="O71" s="21"/>
     </row>
     <row r="72" customFormat="false" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A72" s="28"/>
+      <c r="A72" s="27"/>
       <c r="B72" s="19"/>
       <c r="C72" s="19"/>
       <c r="D72" s="19"/>
@@ -5531,7 +5521,7 @@
       <c r="F72" s="18"/>
       <c r="G72" s="18"/>
       <c r="H72" s="18"/>
-      <c r="I72" s="24" t="s">
+      <c r="I72" s="23" t="s">
         <v>178</v>
       </c>
       <c r="J72" s="21"/>
@@ -5542,7 +5532,7 @@
       <c r="O72" s="21"/>
     </row>
     <row r="73" customFormat="false" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A73" s="28"/>
+      <c r="A73" s="27"/>
       <c r="B73" s="19"/>
       <c r="C73" s="19"/>
       <c r="D73" s="19"/>
@@ -5550,7 +5540,7 @@
       <c r="F73" s="18"/>
       <c r="G73" s="18"/>
       <c r="H73" s="18"/>
-      <c r="I73" s="24" t="s">
+      <c r="I73" s="23" t="s">
         <v>179</v>
       </c>
       <c r="J73" s="21"/>
@@ -5561,7 +5551,7 @@
       <c r="O73" s="21"/>
     </row>
     <row r="74" customFormat="false" ht="39.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A74" s="28"/>
+      <c r="A74" s="27"/>
       <c r="B74" s="19"/>
       <c r="C74" s="19"/>
       <c r="D74" s="19"/>
@@ -5592,13 +5582,13 @@
       <c r="M74" s="21" t="n">
         <v>5</v>
       </c>
-      <c r="N74" s="22" t="s">
+      <c r="N74" s="21" t="s">
         <v>45</v>
       </c>
       <c r="O74" s="21"/>
     </row>
     <row r="75" customFormat="false" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A75" s="28"/>
+      <c r="A75" s="27"/>
       <c r="B75" s="19"/>
       <c r="C75" s="19"/>
       <c r="D75" s="19"/>
@@ -5617,7 +5607,7 @@
       <c r="O75" s="21"/>
     </row>
     <row r="76" customFormat="false" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A76" s="28"/>
+      <c r="A76" s="27"/>
       <c r="B76" s="19"/>
       <c r="C76" s="19"/>
       <c r="D76" s="19"/>
@@ -5636,7 +5626,7 @@
       <c r="O76" s="21"/>
     </row>
     <row r="77" customFormat="false" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A77" s="28"/>
+      <c r="A77" s="27"/>
       <c r="B77" s="19"/>
       <c r="C77" s="19"/>
       <c r="D77" s="19"/>
@@ -5655,7 +5645,7 @@
       <c r="O77" s="21"/>
     </row>
     <row r="78" customFormat="false" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A78" s="28"/>
+      <c r="A78" s="27"/>
       <c r="B78" s="19"/>
       <c r="C78" s="19"/>
       <c r="D78" s="19"/>
@@ -5663,7 +5653,7 @@
       <c r="F78" s="18"/>
       <c r="G78" s="18"/>
       <c r="H78" s="18"/>
-      <c r="I78" s="24" t="s">
+      <c r="I78" s="23" t="s">
         <v>189</v>
       </c>
       <c r="J78" s="21"/>
@@ -5673,8 +5663,8 @@
       <c r="N78" s="21"/>
       <c r="O78" s="21"/>
     </row>
-    <row r="79" s="29" customFormat="true" ht="39.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A79" s="28"/>
+    <row r="79" s="28" customFormat="true" ht="39.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A79" s="27"/>
       <c r="B79" s="19"/>
       <c r="C79" s="19"/>
       <c r="D79" s="19"/>
@@ -5690,7 +5680,7 @@
       <c r="H79" s="21" t="s">
         <v>193</v>
       </c>
-      <c r="I79" s="24" t="s">
+      <c r="I79" s="23" t="s">
         <v>194</v>
       </c>
       <c r="J79" s="21" t="s">
@@ -5705,7 +5695,7 @@
       <c r="M79" s="21" t="n">
         <v>5</v>
       </c>
-      <c r="N79" s="22" t="s">
+      <c r="N79" s="21" t="s">
         <v>45</v>
       </c>
       <c r="O79" s="21"/>
@@ -5713,7 +5703,7 @@
       <c r="XFD79" s="1"/>
     </row>
     <row r="80" customFormat="false" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A80" s="28"/>
+      <c r="A80" s="27"/>
       <c r="B80" s="19"/>
       <c r="C80" s="19"/>
       <c r="D80" s="19"/>
@@ -5721,7 +5711,7 @@
       <c r="F80" s="17"/>
       <c r="G80" s="17"/>
       <c r="H80" s="17"/>
-      <c r="I80" s="24" t="s">
+      <c r="I80" s="23" t="s">
         <v>196</v>
       </c>
       <c r="J80" s="21"/>
@@ -5732,7 +5722,7 @@
       <c r="O80" s="21"/>
     </row>
     <row r="81" customFormat="false" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A81" s="28"/>
+      <c r="A81" s="27"/>
       <c r="B81" s="19"/>
       <c r="C81" s="19"/>
       <c r="D81" s="19"/>
@@ -5740,7 +5730,7 @@
       <c r="F81" s="17"/>
       <c r="G81" s="17"/>
       <c r="H81" s="17"/>
-      <c r="I81" s="24" t="s">
+      <c r="I81" s="23" t="s">
         <v>197</v>
       </c>
       <c r="J81" s="21"/>
@@ -5751,7 +5741,7 @@
       <c r="O81" s="21"/>
     </row>
     <row r="82" customFormat="false" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A82" s="28"/>
+      <c r="A82" s="27"/>
       <c r="B82" s="19"/>
       <c r="C82" s="19"/>
       <c r="D82" s="19"/>
@@ -5759,7 +5749,7 @@
       <c r="F82" s="17"/>
       <c r="G82" s="17"/>
       <c r="H82" s="17"/>
-      <c r="I82" s="24" t="s">
+      <c r="I82" s="23" t="s">
         <v>198</v>
       </c>
       <c r="J82" s="21"/>
@@ -5770,7 +5760,7 @@
       <c r="O82" s="21"/>
     </row>
     <row r="83" customFormat="false" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A83" s="28"/>
+      <c r="A83" s="27"/>
       <c r="B83" s="19"/>
       <c r="C83" s="19"/>
       <c r="D83" s="19"/>
@@ -5778,7 +5768,7 @@
       <c r="F83" s="17"/>
       <c r="G83" s="17"/>
       <c r="H83" s="17"/>
-      <c r="I83" s="24" t="s">
+      <c r="I83" s="23" t="s">
         <v>199</v>
       </c>
       <c r="J83" s="21"/>
@@ -5789,7 +5779,7 @@
       <c r="O83" s="21"/>
     </row>
     <row r="84" customFormat="false" ht="39.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A84" s="28"/>
+      <c r="A84" s="27"/>
       <c r="B84" s="19"/>
       <c r="C84" s="19"/>
       <c r="D84" s="19"/>
@@ -5805,7 +5795,7 @@
       <c r="H84" s="21" t="s">
         <v>202</v>
       </c>
-      <c r="I84" s="24" t="s">
+      <c r="I84" s="23" t="s">
         <v>203</v>
       </c>
       <c r="J84" s="21" t="s">
@@ -5820,13 +5810,13 @@
       <c r="M84" s="21" t="n">
         <v>5</v>
       </c>
-      <c r="N84" s="22" t="s">
+      <c r="N84" s="21" t="s">
         <v>45</v>
       </c>
       <c r="O84" s="21"/>
     </row>
     <row r="85" customFormat="false" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A85" s="28"/>
+      <c r="A85" s="27"/>
       <c r="B85" s="19"/>
       <c r="C85" s="19"/>
       <c r="D85" s="19"/>
@@ -5834,7 +5824,7 @@
       <c r="F85" s="17"/>
       <c r="G85" s="17"/>
       <c r="H85" s="17"/>
-      <c r="I85" s="24" t="s">
+      <c r="I85" s="23" t="s">
         <v>204</v>
       </c>
       <c r="J85" s="21"/>
@@ -5845,7 +5835,7 @@
       <c r="O85" s="21"/>
     </row>
     <row r="86" customFormat="false" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A86" s="28"/>
+      <c r="A86" s="27"/>
       <c r="B86" s="19"/>
       <c r="C86" s="19"/>
       <c r="D86" s="19"/>
@@ -5853,7 +5843,7 @@
       <c r="F86" s="17"/>
       <c r="G86" s="17"/>
       <c r="H86" s="17"/>
-      <c r="I86" s="24" t="s">
+      <c r="I86" s="23" t="s">
         <v>205</v>
       </c>
       <c r="J86" s="21"/>
@@ -5864,7 +5854,7 @@
       <c r="O86" s="21"/>
     </row>
     <row r="87" customFormat="false" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A87" s="28"/>
+      <c r="A87" s="27"/>
       <c r="B87" s="19"/>
       <c r="C87" s="19"/>
       <c r="D87" s="19"/>
@@ -5872,7 +5862,7 @@
       <c r="F87" s="17"/>
       <c r="G87" s="17"/>
       <c r="H87" s="17"/>
-      <c r="I87" s="24" t="s">
+      <c r="I87" s="23" t="s">
         <v>206</v>
       </c>
       <c r="J87" s="21"/>
@@ -5883,7 +5873,7 @@
       <c r="O87" s="21"/>
     </row>
     <row r="88" customFormat="false" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A88" s="28"/>
+      <c r="A88" s="27"/>
       <c r="B88" s="19"/>
       <c r="C88" s="19"/>
       <c r="D88" s="19"/>
@@ -5891,7 +5881,7 @@
       <c r="F88" s="17"/>
       <c r="G88" s="17"/>
       <c r="H88" s="17"/>
-      <c r="I88" s="24" t="s">
+      <c r="I88" s="23" t="s">
         <v>198</v>
       </c>
       <c r="J88" s="21"/>
@@ -5902,7 +5892,7 @@
       <c r="O88" s="21"/>
     </row>
     <row r="89" customFormat="false" ht="39.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A89" s="28"/>
+      <c r="A89" s="27"/>
       <c r="B89" s="19"/>
       <c r="C89" s="19"/>
       <c r="D89" s="19"/>
@@ -5918,7 +5908,7 @@
       <c r="H89" s="21" t="s">
         <v>209</v>
       </c>
-      <c r="I89" s="24" t="s">
+      <c r="I89" s="23" t="s">
         <v>210</v>
       </c>
       <c r="J89" s="21" t="s">
@@ -5933,13 +5923,13 @@
       <c r="M89" s="21" t="n">
         <v>1</v>
       </c>
-      <c r="N89" s="22" t="s">
+      <c r="N89" s="21" t="s">
         <v>45</v>
       </c>
       <c r="O89" s="21"/>
     </row>
     <row r="90" customFormat="false" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A90" s="28"/>
+      <c r="A90" s="27"/>
       <c r="B90" s="19"/>
       <c r="C90" s="19"/>
       <c r="D90" s="19"/>
@@ -5947,7 +5937,7 @@
       <c r="F90" s="21"/>
       <c r="G90" s="21"/>
       <c r="H90" s="21"/>
-      <c r="I90" s="24" t="s">
+      <c r="I90" s="23" t="s">
         <v>212</v>
       </c>
       <c r="J90" s="21"/>
@@ -5958,7 +5948,7 @@
       <c r="O90" s="21"/>
     </row>
     <row r="91" customFormat="false" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A91" s="28"/>
+      <c r="A91" s="27"/>
       <c r="B91" s="19"/>
       <c r="C91" s="19"/>
       <c r="D91" s="19"/>
@@ -5966,7 +5956,7 @@
       <c r="F91" s="21"/>
       <c r="G91" s="21"/>
       <c r="H91" s="21"/>
-      <c r="I91" s="24" t="s">
+      <c r="I91" s="23" t="s">
         <v>213</v>
       </c>
       <c r="J91" s="21"/>
@@ -5977,7 +5967,7 @@
       <c r="O91" s="21"/>
     </row>
     <row r="92" customFormat="false" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A92" s="28"/>
+      <c r="A92" s="27"/>
       <c r="B92" s="19"/>
       <c r="C92" s="19"/>
       <c r="D92" s="19"/>
@@ -5985,7 +5975,7 @@
       <c r="F92" s="21"/>
       <c r="G92" s="21"/>
       <c r="H92" s="21"/>
-      <c r="I92" s="24" t="s">
+      <c r="I92" s="23" t="s">
         <v>198</v>
       </c>
       <c r="J92" s="21"/>
@@ -5996,7 +5986,7 @@
       <c r="O92" s="21"/>
     </row>
     <row r="93" customFormat="false" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A93" s="28"/>
+      <c r="A93" s="27"/>
       <c r="B93" s="19"/>
       <c r="C93" s="19"/>
       <c r="D93" s="19"/>
@@ -6004,7 +5994,7 @@
       <c r="F93" s="21"/>
       <c r="G93" s="21"/>
       <c r="H93" s="21"/>
-      <c r="I93" s="24" t="s">
+      <c r="I93" s="23" t="s">
         <v>214</v>
       </c>
       <c r="J93" s="21"/>
@@ -6015,7 +6005,7 @@
       <c r="O93" s="21"/>
     </row>
     <row r="94" customFormat="false" ht="35.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A94" s="28"/>
+      <c r="A94" s="27"/>
       <c r="B94" s="19"/>
       <c r="C94" s="19"/>
       <c r="D94" s="19"/>
@@ -6031,7 +6021,7 @@
       <c r="H94" s="21" t="s">
         <v>218</v>
       </c>
-      <c r="I94" s="24" t="s">
+      <c r="I94" s="23" t="s">
         <v>219</v>
       </c>
       <c r="J94" s="21" t="s">
@@ -6046,13 +6036,13 @@
       <c r="M94" s="21" t="n">
         <v>1</v>
       </c>
-      <c r="N94" s="22" t="s">
+      <c r="N94" s="21" t="s">
         <v>45</v>
       </c>
-      <c r="O94" s="30"/>
+      <c r="O94" s="29"/>
     </row>
     <row r="95" customFormat="false" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A95" s="28"/>
+      <c r="A95" s="27"/>
       <c r="B95" s="19"/>
       <c r="C95" s="19"/>
       <c r="D95" s="19"/>
@@ -6060,7 +6050,7 @@
       <c r="F95" s="21"/>
       <c r="G95" s="21"/>
       <c r="H95" s="21"/>
-      <c r="I95" s="24" t="s">
+      <c r="I95" s="23" t="s">
         <v>220</v>
       </c>
       <c r="J95" s="21"/>
@@ -6071,7 +6061,7 @@
       <c r="O95" s="21"/>
     </row>
     <row r="96" customFormat="false" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A96" s="28"/>
+      <c r="A96" s="27"/>
       <c r="B96" s="19"/>
       <c r="C96" s="19"/>
       <c r="D96" s="19"/>
@@ -6079,7 +6069,7 @@
       <c r="F96" s="21"/>
       <c r="G96" s="21"/>
       <c r="H96" s="21"/>
-      <c r="I96" s="24" t="s">
+      <c r="I96" s="23" t="s">
         <v>221</v>
       </c>
       <c r="J96" s="21"/>
@@ -6090,7 +6080,7 @@
       <c r="O96" s="21"/>
     </row>
     <row r="97" customFormat="false" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A97" s="28"/>
+      <c r="A97" s="27"/>
       <c r="B97" s="19"/>
       <c r="C97" s="19"/>
       <c r="D97" s="19"/>
@@ -6098,7 +6088,7 @@
       <c r="F97" s="21"/>
       <c r="G97" s="21"/>
       <c r="H97" s="21"/>
-      <c r="I97" s="24" t="s">
+      <c r="I97" s="23" t="s">
         <v>222</v>
       </c>
       <c r="J97" s="21"/>
@@ -6109,7 +6099,7 @@
       <c r="O97" s="21"/>
     </row>
     <row r="98" customFormat="false" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A98" s="28"/>
+      <c r="A98" s="27"/>
       <c r="B98" s="19"/>
       <c r="C98" s="19"/>
       <c r="D98" s="19"/>
@@ -6117,7 +6107,7 @@
       <c r="F98" s="21"/>
       <c r="G98" s="21"/>
       <c r="H98" s="21"/>
-      <c r="I98" s="24" t="s">
+      <c r="I98" s="23" t="s">
         <v>223</v>
       </c>
       <c r="J98" s="21"/>
@@ -6128,7 +6118,7 @@
       <c r="O98" s="21"/>
     </row>
     <row r="99" customFormat="false" ht="71.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A99" s="28"/>
+      <c r="A99" s="27"/>
       <c r="B99" s="19"/>
       <c r="C99" s="19"/>
       <c r="D99" s="19"/>
@@ -6144,7 +6134,7 @@
       <c r="H99" s="21" t="s">
         <v>226</v>
       </c>
-      <c r="I99" s="31" t="s">
+      <c r="I99" s="30" t="s">
         <v>227</v>
       </c>
       <c r="J99" s="21" t="s">
@@ -6159,13 +6149,13 @@
       <c r="M99" s="21" t="n">
         <v>2</v>
       </c>
-      <c r="N99" s="22" t="s">
+      <c r="N99" s="21" t="s">
         <v>45</v>
       </c>
       <c r="O99" s="21"/>
     </row>
     <row r="100" customFormat="false" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A100" s="28"/>
+      <c r="A100" s="27"/>
       <c r="B100" s="19"/>
       <c r="C100" s="19"/>
       <c r="D100" s="19"/>
@@ -6173,7 +6163,7 @@
       <c r="F100" s="21"/>
       <c r="G100" s="21"/>
       <c r="H100" s="21"/>
-      <c r="I100" s="31" t="s">
+      <c r="I100" s="30" t="s">
         <v>228</v>
       </c>
       <c r="J100" s="21"/>
@@ -6184,7 +6174,7 @@
       <c r="O100" s="21"/>
     </row>
     <row r="101" customFormat="false" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A101" s="28"/>
+      <c r="A101" s="27"/>
       <c r="B101" s="19"/>
       <c r="C101" s="19"/>
       <c r="D101" s="19"/>
@@ -6192,7 +6182,7 @@
       <c r="F101" s="21"/>
       <c r="G101" s="21"/>
       <c r="H101" s="21"/>
-      <c r="I101" s="32" t="s">
+      <c r="I101" s="31" t="s">
         <v>229</v>
       </c>
       <c r="J101" s="21"/>
@@ -6203,7 +6193,7 @@
       <c r="O101" s="21"/>
     </row>
     <row r="102" customFormat="false" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A102" s="28"/>
+      <c r="A102" s="27"/>
       <c r="B102" s="19"/>
       <c r="C102" s="19"/>
       <c r="D102" s="19"/>
@@ -6211,7 +6201,7 @@
       <c r="F102" s="21"/>
       <c r="G102" s="21"/>
       <c r="H102" s="21"/>
-      <c r="I102" s="31" t="s">
+      <c r="I102" s="30" t="s">
         <v>230</v>
       </c>
       <c r="J102" s="21"/>
@@ -6222,7 +6212,7 @@
       <c r="O102" s="21"/>
     </row>
     <row r="103" customFormat="false" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A103" s="28"/>
+      <c r="A103" s="27"/>
       <c r="B103" s="19"/>
       <c r="C103" s="19"/>
       <c r="D103" s="19"/>
@@ -6230,7 +6220,7 @@
       <c r="F103" s="21"/>
       <c r="G103" s="21"/>
       <c r="H103" s="21"/>
-      <c r="I103" s="32" t="s">
+      <c r="I103" s="31" t="s">
         <v>231</v>
       </c>
       <c r="J103" s="21"/>
@@ -6241,7 +6231,7 @@
       <c r="O103" s="21"/>
     </row>
     <row r="104" customFormat="false" ht="39.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A104" s="33" t="s">
+      <c r="A104" s="32" t="s">
         <v>232</v>
       </c>
       <c r="B104" s="17" t="s">
@@ -6280,13 +6270,13 @@
       <c r="M104" s="21" t="n">
         <v>6</v>
       </c>
-      <c r="N104" s="22" t="s">
+      <c r="N104" s="21" t="s">
         <v>45</v>
       </c>
       <c r="O104" s="21"/>
     </row>
     <row r="105" customFormat="false" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A105" s="33"/>
+      <c r="A105" s="32"/>
       <c r="B105" s="17"/>
       <c r="C105" s="17"/>
       <c r="D105" s="17"/>
@@ -6305,7 +6295,7 @@
       <c r="O105" s="21"/>
     </row>
     <row r="106" customFormat="false" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A106" s="33"/>
+      <c r="A106" s="32"/>
       <c r="B106" s="17"/>
       <c r="C106" s="17"/>
       <c r="D106" s="17"/>
@@ -6324,7 +6314,7 @@
       <c r="O106" s="21"/>
     </row>
     <row r="107" customFormat="false" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A107" s="33"/>
+      <c r="A107" s="32"/>
       <c r="B107" s="17"/>
       <c r="C107" s="17"/>
       <c r="D107" s="17"/>
@@ -6343,7 +6333,7 @@
       <c r="O107" s="21"/>
     </row>
     <row r="108" customFormat="false" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A108" s="33"/>
+      <c r="A108" s="32"/>
       <c r="B108" s="17"/>
       <c r="C108" s="17"/>
       <c r="D108" s="17"/>
@@ -6362,7 +6352,7 @@
       <c r="O108" s="21"/>
     </row>
     <row r="109" customFormat="false" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A109" s="33"/>
+      <c r="A109" s="32"/>
       <c r="B109" s="17"/>
       <c r="C109" s="17"/>
       <c r="D109" s="17"/>
@@ -6370,7 +6360,7 @@
       <c r="F109" s="19"/>
       <c r="G109" s="19"/>
       <c r="H109" s="20"/>
-      <c r="I109" s="24" t="s">
+      <c r="I109" s="23" t="s">
         <v>245</v>
       </c>
       <c r="J109" s="21"/>
@@ -6381,7 +6371,7 @@
       <c r="O109" s="21"/>
     </row>
     <row r="110" customFormat="false" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A110" s="33"/>
+      <c r="A110" s="32"/>
       <c r="B110" s="17"/>
       <c r="C110" s="17"/>
       <c r="D110" s="17"/>
@@ -6400,7 +6390,7 @@
       <c r="O110" s="21"/>
     </row>
     <row r="111" customFormat="false" ht="52" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A111" s="33"/>
+      <c r="A111" s="32"/>
       <c r="B111" s="17"/>
       <c r="C111" s="17"/>
       <c r="D111" s="17"/>
@@ -6431,13 +6421,13 @@
       <c r="M111" s="21" t="n">
         <v>6</v>
       </c>
-      <c r="N111" s="22" t="s">
+      <c r="N111" s="21" t="s">
         <v>45</v>
       </c>
       <c r="O111" s="21"/>
     </row>
     <row r="112" customFormat="false" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A112" s="33"/>
+      <c r="A112" s="32"/>
       <c r="B112" s="17"/>
       <c r="C112" s="17"/>
       <c r="D112" s="17"/>
@@ -6456,7 +6446,7 @@
       <c r="O112" s="21"/>
     </row>
     <row r="113" customFormat="false" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A113" s="33"/>
+      <c r="A113" s="32"/>
       <c r="B113" s="17"/>
       <c r="C113" s="17"/>
       <c r="D113" s="17"/>
@@ -6475,7 +6465,7 @@
       <c r="O113" s="21"/>
     </row>
     <row r="114" customFormat="false" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A114" s="33"/>
+      <c r="A114" s="32"/>
       <c r="B114" s="17"/>
       <c r="C114" s="17"/>
       <c r="D114" s="17"/>
@@ -6494,7 +6484,7 @@
       <c r="O114" s="21"/>
     </row>
     <row r="115" customFormat="false" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A115" s="33"/>
+      <c r="A115" s="32"/>
       <c r="B115" s="17"/>
       <c r="C115" s="17"/>
       <c r="D115" s="17"/>
@@ -6513,7 +6503,7 @@
       <c r="O115" s="21"/>
     </row>
     <row r="116" customFormat="false" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A116" s="33"/>
+      <c r="A116" s="32"/>
       <c r="B116" s="17"/>
       <c r="C116" s="17"/>
       <c r="D116" s="17"/>
@@ -6521,7 +6511,7 @@
       <c r="F116" s="17"/>
       <c r="G116" s="17"/>
       <c r="H116" s="17"/>
-      <c r="I116" s="24" t="s">
+      <c r="I116" s="23" t="s">
         <v>256</v>
       </c>
       <c r="J116" s="21"/>
@@ -6532,7 +6522,7 @@
       <c r="O116" s="21"/>
     </row>
     <row r="117" customFormat="false" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A117" s="33"/>
+      <c r="A117" s="32"/>
       <c r="B117" s="17"/>
       <c r="C117" s="17"/>
       <c r="D117" s="17"/>
@@ -6551,7 +6541,7 @@
       <c r="O117" s="21"/>
     </row>
     <row r="118" customFormat="false" ht="99.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A118" s="33"/>
+      <c r="A118" s="32"/>
       <c r="B118" s="17"/>
       <c r="C118" s="17"/>
       <c r="D118" s="17"/>
@@ -6582,13 +6572,13 @@
       <c r="M118" s="21" t="n">
         <v>6</v>
       </c>
-      <c r="N118" s="22" t="s">
+      <c r="N118" s="21" t="s">
         <v>45</v>
       </c>
       <c r="O118" s="21"/>
     </row>
     <row r="119" customFormat="false" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A119" s="33"/>
+      <c r="A119" s="32"/>
       <c r="B119" s="17"/>
       <c r="C119" s="17"/>
       <c r="D119" s="17"/>
@@ -6607,7 +6597,7 @@
       <c r="O119" s="21"/>
     </row>
     <row r="120" customFormat="false" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A120" s="33"/>
+      <c r="A120" s="32"/>
       <c r="B120" s="17"/>
       <c r="C120" s="17"/>
       <c r="D120" s="17"/>
@@ -6626,7 +6616,7 @@
       <c r="O120" s="21"/>
     </row>
     <row r="121" customFormat="false" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A121" s="33"/>
+      <c r="A121" s="32"/>
       <c r="B121" s="17"/>
       <c r="C121" s="17"/>
       <c r="D121" s="17"/>
@@ -6645,7 +6635,7 @@
       <c r="O121" s="21"/>
     </row>
     <row r="122" customFormat="false" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A122" s="33"/>
+      <c r="A122" s="32"/>
       <c r="B122" s="17"/>
       <c r="C122" s="17"/>
       <c r="D122" s="17"/>
@@ -6664,7 +6654,7 @@
       <c r="O122" s="21"/>
     </row>
     <row r="123" customFormat="false" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A123" s="33"/>
+      <c r="A123" s="32"/>
       <c r="B123" s="17"/>
       <c r="C123" s="17"/>
       <c r="D123" s="17"/>
@@ -6683,7 +6673,7 @@
       <c r="O123" s="21"/>
     </row>
     <row r="124" customFormat="false" ht="52" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A124" s="33"/>
+      <c r="A124" s="32"/>
       <c r="B124" s="17"/>
       <c r="C124" s="17"/>
       <c r="D124" s="17"/>
@@ -6714,13 +6704,13 @@
       <c r="M124" s="21" t="n">
         <v>6</v>
       </c>
-      <c r="N124" s="22" t="s">
+      <c r="N124" s="21" t="s">
         <v>45</v>
       </c>
       <c r="O124" s="21"/>
     </row>
     <row r="125" customFormat="false" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A125" s="33"/>
+      <c r="A125" s="32"/>
       <c r="B125" s="17"/>
       <c r="C125" s="17"/>
       <c r="D125" s="17"/>
@@ -6739,7 +6729,7 @@
       <c r="O125" s="21"/>
     </row>
     <row r="126" customFormat="false" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A126" s="33"/>
+      <c r="A126" s="32"/>
       <c r="B126" s="17"/>
       <c r="C126" s="17"/>
       <c r="D126" s="17"/>
@@ -6747,7 +6737,7 @@
       <c r="F126" s="19"/>
       <c r="G126" s="19"/>
       <c r="H126" s="19"/>
-      <c r="I126" s="24" t="s">
+      <c r="I126" s="23" t="s">
         <v>271</v>
       </c>
       <c r="J126" s="21"/>
@@ -6758,7 +6748,7 @@
       <c r="O126" s="21"/>
     </row>
     <row r="127" customFormat="false" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A127" s="33"/>
+      <c r="A127" s="32"/>
       <c r="B127" s="17"/>
       <c r="C127" s="17"/>
       <c r="D127" s="17"/>
@@ -6776,8 +6766,8 @@
       <c r="N127" s="21"/>
       <c r="O127" s="21"/>
     </row>
-    <row r="128" s="35" customFormat="true" ht="52" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A128" s="34" t="s">
+    <row r="128" s="34" customFormat="true" ht="52" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A128" s="33" t="s">
         <v>273</v>
       </c>
       <c r="B128" s="17" t="s">
@@ -6816,15 +6806,15 @@
       <c r="M128" s="21" t="n">
         <v>3</v>
       </c>
-      <c r="N128" s="22" t="s">
+      <c r="N128" s="21" t="s">
         <v>45</v>
       </c>
       <c r="O128" s="21"/>
       <c r="XFC128" s="3"/>
       <c r="XFD128" s="1"/>
     </row>
-    <row r="129" s="36" customFormat="true" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A129" s="34"/>
+    <row r="129" s="35" customFormat="true" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A129" s="33"/>
       <c r="B129" s="17"/>
       <c r="C129" s="17"/>
       <c r="D129" s="17"/>
@@ -6844,8 +6834,8 @@
       <c r="XFC129" s="3"/>
       <c r="XFD129" s="1"/>
     </row>
-    <row r="130" s="36" customFormat="true" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A130" s="34"/>
+    <row r="130" s="35" customFormat="true" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A130" s="33"/>
       <c r="B130" s="17"/>
       <c r="C130" s="17"/>
       <c r="D130" s="17"/>
@@ -6865,8 +6855,8 @@
       <c r="XFC130" s="3"/>
       <c r="XFD130" s="1"/>
     </row>
-    <row r="131" s="36" customFormat="true" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A131" s="34"/>
+    <row r="131" s="35" customFormat="true" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A131" s="33"/>
       <c r="B131" s="17"/>
       <c r="C131" s="17"/>
       <c r="D131" s="17"/>
@@ -6886,8 +6876,8 @@
       <c r="XFC131" s="3"/>
       <c r="XFD131" s="1"/>
     </row>
-    <row r="132" s="36" customFormat="true" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A132" s="34"/>
+    <row r="132" s="35" customFormat="true" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A132" s="33"/>
       <c r="B132" s="17"/>
       <c r="C132" s="17"/>
       <c r="D132" s="17"/>
@@ -6907,8 +6897,8 @@
       <c r="XFC132" s="3"/>
       <c r="XFD132" s="1"/>
     </row>
-    <row r="133" s="36" customFormat="true" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A133" s="34"/>
+    <row r="133" s="35" customFormat="true" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A133" s="33"/>
       <c r="B133" s="17"/>
       <c r="C133" s="17"/>
       <c r="D133" s="17"/>
@@ -6928,8 +6918,8 @@
       <c r="XFC133" s="3"/>
       <c r="XFD133" s="1"/>
     </row>
-    <row r="134" s="36" customFormat="true" ht="39.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A134" s="34"/>
+    <row r="134" s="35" customFormat="true" ht="39.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A134" s="33"/>
       <c r="B134" s="17"/>
       <c r="C134" s="17"/>
       <c r="D134" s="17"/>
@@ -6960,15 +6950,15 @@
       <c r="M134" s="21" t="n">
         <v>7</v>
       </c>
-      <c r="N134" s="22" t="s">
+      <c r="N134" s="21" t="s">
         <v>45</v>
       </c>
       <c r="O134" s="21"/>
       <c r="XFC134" s="3"/>
       <c r="XFD134" s="1"/>
     </row>
-    <row r="135" s="36" customFormat="true" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A135" s="34"/>
+    <row r="135" s="35" customFormat="true" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A135" s="33"/>
       <c r="B135" s="17"/>
       <c r="C135" s="17"/>
       <c r="D135" s="17"/>
@@ -6988,8 +6978,8 @@
       <c r="XFC135" s="3"/>
       <c r="XFD135" s="1"/>
     </row>
-    <row r="136" s="36" customFormat="true" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A136" s="34"/>
+    <row r="136" s="35" customFormat="true" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A136" s="33"/>
       <c r="B136" s="17"/>
       <c r="C136" s="17"/>
       <c r="D136" s="17"/>
@@ -7009,8 +6999,8 @@
       <c r="XFC136" s="3"/>
       <c r="XFD136" s="1"/>
     </row>
-    <row r="137" s="36" customFormat="true" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A137" s="34"/>
+    <row r="137" s="35" customFormat="true" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A137" s="33"/>
       <c r="B137" s="17"/>
       <c r="C137" s="17"/>
       <c r="D137" s="17"/>
@@ -7030,8 +7020,8 @@
       <c r="XFC137" s="3"/>
       <c r="XFD137" s="1"/>
     </row>
-    <row r="138" s="36" customFormat="true" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A138" s="34"/>
+    <row r="138" s="35" customFormat="true" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A138" s="33"/>
       <c r="B138" s="17"/>
       <c r="C138" s="17"/>
       <c r="D138" s="17"/>
@@ -7051,8 +7041,8 @@
       <c r="XFC138" s="3"/>
       <c r="XFD138" s="1"/>
     </row>
-    <row r="139" s="36" customFormat="true" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A139" s="34"/>
+    <row r="139" s="35" customFormat="true" ht="99.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A139" s="33"/>
       <c r="B139" s="17"/>
       <c r="C139" s="17"/>
       <c r="D139" s="17"/>
@@ -7458,13 +7448,13 @@
   <sheetData>
     <row r="1" customFormat="false" ht="71.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="2" s="1" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="37"/>
-      <c r="B2" s="37"/>
-      <c r="C2" s="37"/>
-      <c r="D2" s="37"/>
-      <c r="E2" s="37"/>
-      <c r="F2" s="37"/>
-      <c r="G2" s="37"/>
+      <c r="A2" s="36"/>
+      <c r="B2" s="36"/>
+      <c r="C2" s="36"/>
+      <c r="D2" s="36"/>
+      <c r="E2" s="36"/>
+      <c r="F2" s="36"/>
+      <c r="G2" s="36"/>
     </row>
     <row r="3" s="1" customFormat="true" ht="14.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="9" t="s">
@@ -7484,71 +7474,71 @@
       <c r="A5" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="24" t="s">
+      <c r="B5" s="23" t="s">
         <v>1</v>
       </c>
-      <c r="C5" s="24"/>
-      <c r="D5" s="24"/>
+      <c r="C5" s="23"/>
+      <c r="D5" s="23"/>
     </row>
     <row r="6" s="1" customFormat="true" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="B6" s="24" t="s">
+      <c r="B6" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="C6" s="24"/>
-      <c r="D6" s="24"/>
+      <c r="C6" s="23"/>
+      <c r="D6" s="23"/>
     </row>
     <row r="7" s="1" customFormat="true" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B7" s="24" t="s">
+      <c r="B7" s="23" t="s">
         <v>5</v>
       </c>
-      <c r="C7" s="24"/>
-      <c r="D7" s="24"/>
+      <c r="C7" s="23"/>
+      <c r="D7" s="23"/>
     </row>
     <row r="8" s="1" customFormat="true" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="24" t="s">
+      <c r="B8" s="23" t="s">
         <v>7</v>
       </c>
-      <c r="C8" s="24"/>
-      <c r="D8" s="24"/>
+      <c r="C8" s="23"/>
+      <c r="D8" s="23"/>
     </row>
     <row r="9" s="1" customFormat="true" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="24" t="s">
+      <c r="B9" s="23" t="s">
         <v>9</v>
       </c>
-      <c r="C9" s="24"/>
-      <c r="D9" s="24"/>
+      <c r="C9" s="23"/>
+      <c r="D9" s="23"/>
     </row>
     <row r="10" s="1" customFormat="true" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="B10" s="24" t="s">
+      <c r="B10" s="23" t="s">
         <v>11</v>
       </c>
-      <c r="C10" s="24"/>
-      <c r="D10" s="24"/>
+      <c r="C10" s="23"/>
+      <c r="D10" s="23"/>
     </row>
     <row r="11" s="1" customFormat="true" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="B11" s="24" t="s">
+      <c r="B11" s="23" t="s">
         <v>13</v>
       </c>
-      <c r="C11" s="24"/>
-      <c r="D11" s="24"/>
+      <c r="C11" s="23"/>
+      <c r="D11" s="23"/>
     </row>
     <row r="12" s="1" customFormat="true" ht="50.55" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
@@ -7559,56 +7549,56 @@
       </c>
       <c r="C12" s="8"/>
       <c r="D12" s="8"/>
-      <c r="E12" s="38"/>
+      <c r="E12" s="37"/>
     </row>
     <row r="13" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="B13" s="24" t="s">
+      <c r="B13" s="23" t="s">
         <v>17</v>
       </c>
-      <c r="C13" s="24"/>
-      <c r="D13" s="24"/>
+      <c r="C13" s="23"/>
+      <c r="D13" s="23"/>
       <c r="E13" s="1"/>
       <c r="F13" s="1"/>
       <c r="G13" s="1"/>
     </row>
     <row r="15" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="39" t="s">
+      <c r="A15" s="38" t="s">
         <v>298</v>
       </c>
-      <c r="B15" s="39"/>
-      <c r="C15" s="39"/>
-      <c r="D15" s="39"/>
-      <c r="E15" s="39"/>
-      <c r="F15" s="39"/>
-      <c r="G15" s="39"/>
+      <c r="B15" s="38"/>
+      <c r="C15" s="38"/>
+      <c r="D15" s="38"/>
+      <c r="E15" s="38"/>
+      <c r="F15" s="38"/>
+      <c r="G15" s="38"/>
     </row>
     <row r="16" customFormat="false" ht="27" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="40" t="s">
+      <c r="A16" s="39" t="s">
         <v>299</v>
       </c>
-      <c r="B16" s="40" t="s">
+      <c r="B16" s="39" t="s">
         <v>300</v>
       </c>
-      <c r="C16" s="40" t="s">
+      <c r="C16" s="39" t="s">
         <v>301</v>
       </c>
-      <c r="D16" s="40" t="s">
+      <c r="D16" s="39" t="s">
         <v>302</v>
       </c>
-      <c r="E16" s="41" t="s">
+      <c r="E16" s="40" t="s">
         <v>303</v>
       </c>
-      <c r="F16" s="41" t="s">
+      <c r="F16" s="40" t="s">
         <v>304</v>
       </c>
-      <c r="G16" s="41" t="s">
+      <c r="G16" s="40" t="s">
         <v>305</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="64.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="62.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
         <v>306</v>
       </c>
@@ -7618,16 +7608,16 @@
       <c r="C17" s="6" t="s">
         <v>308</v>
       </c>
-      <c r="D17" s="24" t="s">
+      <c r="D17" s="23" t="s">
         <v>309</v>
       </c>
-      <c r="E17" s="24" t="s">
+      <c r="E17" s="23" t="s">
         <v>310</v>
       </c>
-      <c r="F17" s="24" t="s">
+      <c r="F17" s="23" t="s">
         <v>311</v>
       </c>
-      <c r="G17" s="24" t="s">
+      <c r="G17" s="23" t="s">
         <v>312</v>
       </c>
     </row>
@@ -7641,16 +7631,16 @@
       <c r="C18" s="6" t="s">
         <v>308</v>
       </c>
-      <c r="D18" s="24" t="s">
+      <c r="D18" s="23" t="s">
         <v>315</v>
       </c>
-      <c r="E18" s="24" t="s">
+      <c r="E18" s="23" t="s">
         <v>316</v>
       </c>
-      <c r="F18" s="24" t="s">
+      <c r="F18" s="23" t="s">
         <v>317</v>
       </c>
-      <c r="G18" s="24" t="s">
+      <c r="G18" s="23" t="s">
         <v>318</v>
       </c>
     </row>
@@ -7664,16 +7654,16 @@
       <c r="C19" s="6" t="s">
         <v>308</v>
       </c>
-      <c r="D19" s="24" t="s">
+      <c r="D19" s="23" t="s">
         <v>321</v>
       </c>
-      <c r="E19" s="24" t="s">
+      <c r="E19" s="23" t="s">
         <v>322</v>
       </c>
-      <c r="F19" s="24" t="s">
+      <c r="F19" s="23" t="s">
         <v>323</v>
       </c>
-      <c r="G19" s="24" t="s">
+      <c r="G19" s="23" t="s">
         <v>324</v>
       </c>
     </row>
@@ -7687,16 +7677,16 @@
       <c r="C20" s="6" t="s">
         <v>308</v>
       </c>
-      <c r="D20" s="24" t="s">
+      <c r="D20" s="23" t="s">
         <v>327</v>
       </c>
-      <c r="E20" s="24" t="s">
+      <c r="E20" s="23" t="s">
         <v>328</v>
       </c>
-      <c r="F20" s="24" t="s">
+      <c r="F20" s="23" t="s">
         <v>329</v>
       </c>
-      <c r="G20" s="24" t="s">
+      <c r="G20" s="23" t="s">
         <v>330</v>
       </c>
     </row>
@@ -7710,16 +7700,16 @@
       <c r="C21" s="6" t="s">
         <v>308</v>
       </c>
-      <c r="D21" s="24" t="s">
+      <c r="D21" s="23" t="s">
         <v>333</v>
       </c>
-      <c r="E21" s="24" t="s">
+      <c r="E21" s="23" t="s">
         <v>334</v>
       </c>
-      <c r="F21" s="24" t="s">
+      <c r="F21" s="23" t="s">
         <v>335</v>
       </c>
-      <c r="G21" s="24" t="s">
+      <c r="G21" s="23" t="s">
         <v>336</v>
       </c>
     </row>
@@ -7733,16 +7723,16 @@
       <c r="C22" s="6" t="s">
         <v>308</v>
       </c>
-      <c r="D22" s="24" t="s">
+      <c r="D22" s="23" t="s">
         <v>339</v>
       </c>
-      <c r="E22" s="24" t="s">
+      <c r="E22" s="23" t="s">
         <v>340</v>
       </c>
-      <c r="F22" s="24" t="s">
+      <c r="F22" s="23" t="s">
         <v>341</v>
       </c>
-      <c r="G22" s="24" t="s">
+      <c r="G22" s="23" t="s">
         <v>342</v>
       </c>
     </row>
@@ -7756,16 +7746,16 @@
       <c r="C23" s="6" t="s">
         <v>308</v>
       </c>
-      <c r="D23" s="24" t="s">
+      <c r="D23" s="23" t="s">
         <v>345</v>
       </c>
-      <c r="E23" s="24" t="s">
+      <c r="E23" s="23" t="s">
         <v>346</v>
       </c>
-      <c r="F23" s="24" t="s">
+      <c r="F23" s="23" t="s">
         <v>347</v>
       </c>
-      <c r="G23" s="24" t="s">
+      <c r="G23" s="23" t="s">
         <v>348</v>
       </c>
     </row>
@@ -7779,16 +7769,16 @@
       <c r="C24" s="6" t="s">
         <v>308</v>
       </c>
-      <c r="D24" s="24" t="s">
+      <c r="D24" s="23" t="s">
         <v>351</v>
       </c>
-      <c r="E24" s="24" t="s">
+      <c r="E24" s="23" t="s">
         <v>352</v>
       </c>
-      <c r="F24" s="24" t="s">
+      <c r="F24" s="23" t="s">
         <v>353</v>
       </c>
-      <c r="G24" s="24" t="s">
+      <c r="G24" s="23" t="s">
         <v>354</v>
       </c>
     </row>
@@ -7802,16 +7792,16 @@
       <c r="C25" s="6" t="s">
         <v>357</v>
       </c>
-      <c r="D25" s="24" t="s">
+      <c r="D25" s="23" t="s">
         <v>358</v>
       </c>
-      <c r="E25" s="24" t="s">
+      <c r="E25" s="23" t="s">
         <v>359</v>
       </c>
-      <c r="F25" s="24" t="s">
+      <c r="F25" s="23" t="s">
         <v>360</v>
       </c>
-      <c r="G25" s="24" t="s">
+      <c r="G25" s="23" t="s">
         <v>361</v>
       </c>
     </row>
@@ -7849,236 +7839,236 @@
   <dimension ref="A1:D24"/>
   <sheetFormatPr defaultColWidth="8.42578125" defaultRowHeight="13.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="42" width="29.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="42" width="49.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="42" width="18.71"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16383" min="5" style="42" width="8.42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="42" width="11.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="41" width="29.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="41" width="49.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="41" width="18.71"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16383" min="5" style="41" width="8.42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="41" width="11.53"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="37"/>
-      <c r="B1" s="37"/>
-      <c r="C1" s="37"/>
+      <c r="A1" s="36"/>
+      <c r="B1" s="36"/>
+      <c r="C1" s="36"/>
     </row>
     <row r="2" s="3" customFormat="true" ht="68.2" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="39" t="s">
+      <c r="A2" s="38" t="s">
         <v>362</v>
       </c>
-      <c r="B2" s="39"/>
-      <c r="C2" s="39"/>
-      <c r="D2" s="43"/>
+      <c r="B2" s="38"/>
+      <c r="C2" s="38"/>
+      <c r="D2" s="42"/>
     </row>
     <row r="3" s="3" customFormat="true" ht="5.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="44"/>
-      <c r="D3" s="43"/>
+      <c r="A3" s="43"/>
+      <c r="D3" s="42"/>
     </row>
     <row r="4" s="3" customFormat="true" ht="52.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="45" t="s">
+      <c r="A4" s="44" t="s">
         <v>0</v>
       </c>
       <c r="B4" s="7" t="s">
         <v>1</v>
       </c>
       <c r="C4" s="7"/>
-      <c r="D4" s="43"/>
+      <c r="D4" s="42"/>
     </row>
     <row r="5" s="3" customFormat="true" ht="32.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="45" t="s">
+      <c r="A5" s="44" t="s">
         <v>2</v>
       </c>
       <c r="B5" s="7" t="s">
         <v>3</v>
       </c>
       <c r="C5" s="7"/>
-      <c r="D5" s="43"/>
+      <c r="D5" s="42"/>
     </row>
     <row r="6" s="3" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="45" t="s">
+      <c r="A6" s="44" t="s">
         <v>4</v>
       </c>
       <c r="B6" s="7" t="s">
         <v>5</v>
       </c>
       <c r="C6" s="7"/>
-      <c r="D6" s="43"/>
+      <c r="D6" s="42"/>
     </row>
     <row r="7" s="3" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="45" t="s">
+      <c r="A7" s="44" t="s">
         <v>6</v>
       </c>
       <c r="B7" s="7" t="s">
         <v>7</v>
       </c>
       <c r="C7" s="7"/>
-      <c r="D7" s="43"/>
+      <c r="D7" s="42"/>
     </row>
     <row r="8" s="3" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="45" t="s">
+      <c r="A8" s="44" t="s">
         <v>8</v>
       </c>
       <c r="B8" s="7" t="s">
         <v>9</v>
       </c>
       <c r="C8" s="7"/>
-      <c r="D8" s="43"/>
+      <c r="D8" s="42"/>
     </row>
     <row r="9" s="3" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="45" t="s">
+      <c r="A9" s="44" t="s">
         <v>10</v>
       </c>
       <c r="B9" s="7" t="s">
         <v>11</v>
       </c>
       <c r="C9" s="7"/>
-      <c r="D9" s="43"/>
+      <c r="D9" s="42"/>
     </row>
     <row r="10" s="3" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="45" t="s">
+      <c r="A10" s="44" t="s">
         <v>12</v>
       </c>
       <c r="B10" s="7" t="s">
         <v>13</v>
       </c>
       <c r="C10" s="7"/>
-      <c r="D10" s="43"/>
+      <c r="D10" s="42"/>
     </row>
     <row r="11" s="3" customFormat="true" ht="52" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="45" t="s">
+      <c r="A11" s="44" t="s">
         <v>363</v>
       </c>
       <c r="B11" s="8" t="s">
         <v>15</v>
       </c>
       <c r="C11" s="8"/>
-      <c r="D11" s="43"/>
+      <c r="D11" s="42"/>
     </row>
     <row r="12" s="3" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="45" t="s">
+      <c r="A12" s="44" t="s">
         <v>16</v>
       </c>
       <c r="B12" s="7" t="s">
         <v>17</v>
       </c>
       <c r="C12" s="7"/>
-      <c r="D12" s="43"/>
+      <c r="D12" s="42"/>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="46"/>
-      <c r="B13" s="47"/>
-      <c r="C13" s="47"/>
+      <c r="A13" s="45"/>
+      <c r="B13" s="46"/>
+      <c r="C13" s="46"/>
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="48" t="s">
+      <c r="A14" s="47" t="s">
         <v>364</v>
       </c>
-      <c r="B14" s="48"/>
-      <c r="C14" s="48"/>
+      <c r="B14" s="47"/>
+      <c r="C14" s="47"/>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="42" t="s">
+      <c r="B15" s="41" t="s">
         <v>365</v>
       </c>
-      <c r="C15" s="42" t="s">
+      <c r="C15" s="41" t="s">
         <v>366</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="40" t="s">
+      <c r="A16" s="39" t="s">
         <v>31</v>
       </c>
-      <c r="B16" s="40" t="s">
+      <c r="B16" s="39" t="s">
         <v>367</v>
       </c>
-      <c r="C16" s="49" t="s">
+      <c r="C16" s="48" t="s">
         <v>368</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="29" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="50" t="s">
+      <c r="A17" s="49" t="s">
         <v>369</v>
       </c>
-      <c r="B17" s="51" t="s">
+      <c r="B17" s="50" t="s">
         <v>370</v>
       </c>
-      <c r="C17" s="52" t="n">
+      <c r="C17" s="51" t="n">
         <v>23</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="29" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="50" t="s">
+      <c r="A18" s="49" t="s">
         <v>371</v>
       </c>
-      <c r="B18" s="51" t="s">
+      <c r="B18" s="50" t="s">
         <v>372</v>
       </c>
-      <c r="C18" s="53" t="n">
+      <c r="C18" s="52" t="n">
         <v>26</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="29" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="50" t="s">
+      <c r="A19" s="49" t="s">
         <v>373</v>
       </c>
-      <c r="B19" s="51" t="s">
+      <c r="B19" s="50" t="s">
         <v>374</v>
       </c>
-      <c r="C19" s="53" t="n">
+      <c r="C19" s="52" t="n">
         <v>21</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="29" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="50" t="s">
+      <c r="A20" s="49" t="s">
         <v>375</v>
       </c>
-      <c r="B20" s="51" t="s">
+      <c r="B20" s="50" t="s">
         <v>376</v>
       </c>
-      <c r="C20" s="52" t="n">
+      <c r="C20" s="51" t="n">
         <v>23</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="29" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="50" t="s">
+      <c r="A21" s="49" t="s">
         <v>377</v>
       </c>
-      <c r="B21" s="51" t="s">
+      <c r="B21" s="50" t="s">
         <v>378</v>
       </c>
-      <c r="C21" s="52" t="n">
+      <c r="C21" s="51" t="n">
         <v>20</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="29" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="50" t="s">
+      <c r="A22" s="49" t="s">
         <v>379</v>
       </c>
-      <c r="B22" s="51" t="s">
+      <c r="B22" s="50" t="s">
         <v>380</v>
       </c>
-      <c r="C22" s="52" t="n">
+      <c r="C22" s="51" t="n">
         <v>18</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="50" t="s">
+      <c r="A23" s="49" t="s">
         <v>381</v>
       </c>
-      <c r="B23" s="51" t="s">
+      <c r="B23" s="50" t="s">
         <v>382</v>
       </c>
-      <c r="C23" s="52" t="n">
+      <c r="C23" s="51" t="n">
         <v>8</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="14.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="54" t="s">
+      <c r="A24" s="53" t="s">
         <v>383</v>
       </c>
-      <c r="B24" s="54" t="s">
+      <c r="B24" s="53" t="s">
         <v>384</v>
       </c>
-      <c r="C24" s="55" t="n">
+      <c r="C24" s="54" t="n">
         <f aca="false">SUM(C17:C23)</f>
         <v>139</v>
       </c>

</xml_diff>